<commit_message>
remove descriptions from templates
</commit_message>
<xml_diff>
--- a/templates/Experiments OGM.xlsx
+++ b/templates/Experiments OGM.xlsx
@@ -29,9 +29,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A reference to one or more individuals
-associated to the process
- Select one or more items from
+          <t>Select one or more items from
 Individuals</t>
         </r>
       </text>
@@ -45,10 +43,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>One or more characters used to identify,
-name, or characterize the nature,
-properties, or contents of a sample
- Select one item from Sample identifiers</t>
+          <t>Select one item from Sample identifiers</t>
         </r>
       </text>
     </comment>
@@ -61,10 +56,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>An identifier associated with a
-particular source, used by the data
-provider or owner
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -77,9 +69,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>One or more associations between the
-individual and an organisation.
- Select one or more items from
+          <t>Select one or more items from
 Organisations</t>
         </r>
       </text>
@@ -93,10 +83,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A data field which describes the name of
-the third party company or laboratory
-that provided services.
- Select one item from Organisations</t>
+          <t>Select one item from Organisations</t>
         </r>
       </text>
     </comment>
@@ -109,9 +96,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The number of cells used for DNA
-isolation
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -124,11 +109,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The output of an extraction process in
-which DNA molecules above a molecular
-weight cutoff are purified in order to
-exclude DNA from organellas
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -141,9 +122,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A date field which describes the date on
-which the DNA was isolated from a sample
- DATE (yyyy-mm-dd)</t>
+          <t>DATE (yyyy-mm-dd)</t>
         </r>
       </text>
     </comment>
@@ -156,9 +135,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The quantity of a HMW-DNA per unit
-volume or weight
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -171,8 +148,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The date of the labeling protocol
- DATE (yyyy-mm-dd)</t>
+          <t>DATE (yyyy-mm-dd)</t>
         </r>
       </text>
     </comment>
@@ -185,9 +161,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A protocol description in which input
-nucleic acid material is labeled
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -200,9 +174,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The amount of DNA present in the sample
-after labeling
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -215,11 +187,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The name of the sequencing platform
-(i.e. brand, name of a company that
-produces sequencer equipment). In FAIR
-Genomes: SequencingPlatform.
- Select one item from Sequencing
+          <t>Select one item from Sequencing
 platforms</t>
         </r>
       </text>
@@ -233,11 +201,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The name of the product and model number
-of a manufacturer's genomic (dna)
-sequencer. In FAIR Genomes:
-SequencingInstrumentModel.
- Select one item from Sequencing
+          <t>Select one item from Sequencing
 instrument models</t>
         </r>
       </text>
@@ -251,8 +215,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>When the mapping experiment took place
- DATETIME</t>
+          <t>DATETIME (yyyy-mm-dd hh:mm:ss)</t>
         </r>
       </text>
     </comment>
@@ -265,13 +228,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The unique number assigned to an
-instrument (e.g., a sequencer). This
-could either be the serial number, a
-unique ID generated by the data
-provider/owner, or another character
-string used to identify the instrument
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -284,9 +241,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The instrument (e.g., a sequencer)
-software
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -299,10 +254,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A sequence of characters used to
-uniquely identify a particular
-microassay chip
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -315,9 +267,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The source-specific version of the
-published genome assembly.
- Select one item from Genome accessions</t>
+          <t>Select one item from Genome accessions</t>
         </r>
       </text>
     </comment>
@@ -330,10 +280,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A sequence of characters used to
-uniquely identify a particular run of a
-test on a particular batch of samples
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -346,8 +293,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>An identifier of a submitted job
- STRING_ARRAY: enter one or more values
+          <t>STRING_ARRAY: enter one or more values
 separated by a comma. E.g., 'value
 1','value-2',...</t>
         </r>
@@ -362,9 +308,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The specific version of the Bionano
-Solve software
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -377,9 +321,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The specific version of the Bionano
-Access software
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -392,9 +334,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The total amount of DNA data generated
-during an OGM run
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -407,9 +347,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The molecule N50 for all molecules that
-are ≥ 150 kbp in length
- INTEGER</t>
+          <t>INTEGER</t>
         </r>
       </text>
     </comment>
@@ -422,9 +360,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The molecule N50 for all molecules that
-are ≥ 20 kbp in length
- INTEGER</t>
+          <t>INTEGER</t>
         </r>
       </text>
     </comment>
@@ -437,9 +373,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The average number of fluorescent labels
-per unit length of DNA
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -452,10 +386,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Map rate (%) is the percentage of
-sequencing reads that successfully align
-to a reference genome.
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -468,11 +399,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The percentage of labeled sites whose
-observed positions differ from the
-expected positions in the reference
-genome
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -485,10 +412,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The percentage of expected label sites
-from the reference genome that are
-missing in the observed DNA molecules
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -501,22 +425,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Other NGS quality control metrics,
-including but not limited to (i)
-sequencer metrics such as yield, error
-rate, density (K/mm2), cluster PF (%)
-and phas/prephas (%), (ii) alignment
-metrics such as QM insert size, GC
-content, QM duplicated reads (%), QM
-error rate, uniformity/evenness of
-coverage and maternal cell
-contamination, and (iii) variant call
-metrics such as number of SNVs/CNVs/SVs
-called, number of missense/nonsense
-variants, common variants (%), unique
-variants (%), gender match and trio
-inheritance check
- TEXT</t>
+          <t>TEXT</t>
         </r>
       </text>
     </comment>
@@ -529,10 +438,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Analysis or reanalysis of existing data
-collected by another centre usually for
-a different purpose
- Select one or more items from
+          <t>Select one or more items from
 Organisations</t>
         </r>
       </text>
@@ -546,9 +452,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A written explanation, observation or
-criticism added to textual material
- TEXT</t>
+          <t>TEXT</t>
         </r>
       </text>
     </comment>

</xml_diff>

<commit_message>
chore: remove descriptions from templates (#70)
</commit_message>
<xml_diff>
--- a/templates/Experiments OGM.xlsx
+++ b/templates/Experiments OGM.xlsx
@@ -29,9 +29,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A reference to one or more individuals
-associated to the process
- Select one or more items from
+          <t>Select one or more items from
 Individuals</t>
         </r>
       </text>
@@ -45,10 +43,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>One or more characters used to identify,
-name, or characterize the nature,
-properties, or contents of a sample
- Select one item from Sample identifiers</t>
+          <t>Select one item from Sample identifiers</t>
         </r>
       </text>
     </comment>
@@ -61,10 +56,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>An identifier associated with a
-particular source, used by the data
-provider or owner
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -77,9 +69,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>One or more associations between the
-individual and an organisation.
- Select one or more items from
+          <t>Select one or more items from
 Organisations</t>
         </r>
       </text>
@@ -93,10 +83,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A data field which describes the name of
-the third party company or laboratory
-that provided services.
- Select one item from Organisations</t>
+          <t>Select one item from Organisations</t>
         </r>
       </text>
     </comment>
@@ -109,9 +96,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The number of cells used for DNA
-isolation
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -124,11 +109,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The output of an extraction process in
-which DNA molecules above a molecular
-weight cutoff are purified in order to
-exclude DNA from organellas
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -141,9 +122,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A date field which describes the date on
-which the DNA was isolated from a sample
- DATE (yyyy-mm-dd)</t>
+          <t>DATE (yyyy-mm-dd)</t>
         </r>
       </text>
     </comment>
@@ -156,9 +135,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The quantity of a HMW-DNA per unit
-volume or weight
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -171,8 +148,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The date of the labeling protocol
- DATE (yyyy-mm-dd)</t>
+          <t>DATE (yyyy-mm-dd)</t>
         </r>
       </text>
     </comment>
@@ -185,9 +161,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A protocol description in which input
-nucleic acid material is labeled
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -200,9 +174,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The amount of DNA present in the sample
-after labeling
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -215,11 +187,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The name of the sequencing platform
-(i.e. brand, name of a company that
-produces sequencer equipment). In FAIR
-Genomes: SequencingPlatform.
- Select one item from Sequencing
+          <t>Select one item from Sequencing
 platforms</t>
         </r>
       </text>
@@ -233,11 +201,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The name of the product and model number
-of a manufacturer's genomic (dna)
-sequencer. In FAIR Genomes:
-SequencingInstrumentModel.
- Select one item from Sequencing
+          <t>Select one item from Sequencing
 instrument models</t>
         </r>
       </text>
@@ -251,8 +215,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>When the mapping experiment took place
- DATETIME</t>
+          <t>DATETIME (yyyy-mm-dd hh:mm:ss)</t>
         </r>
       </text>
     </comment>
@@ -265,13 +228,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The unique number assigned to an
-instrument (e.g., a sequencer). This
-could either be the serial number, a
-unique ID generated by the data
-provider/owner, or another character
-string used to identify the instrument
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -284,9 +241,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The instrument (e.g., a sequencer)
-software
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -299,10 +254,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A sequence of characters used to
-uniquely identify a particular
-microassay chip
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -315,9 +267,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The source-specific version of the
-published genome assembly.
- Select one item from Genome accessions</t>
+          <t>Select one item from Genome accessions</t>
         </r>
       </text>
     </comment>
@@ -330,10 +280,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A sequence of characters used to
-uniquely identify a particular run of a
-test on a particular batch of samples
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -346,8 +293,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>An identifier of a submitted job
- STRING_ARRAY: enter one or more values
+          <t>STRING_ARRAY: enter one or more values
 separated by a comma. E.g., 'value
 1','value-2',...</t>
         </r>
@@ -362,9 +308,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The specific version of the Bionano
-Solve software
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -377,9 +321,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The specific version of the Bionano
-Access software
- STRING</t>
+          <t>STRING</t>
         </r>
       </text>
     </comment>
@@ -392,9 +334,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The total amount of DNA data generated
-during an OGM run
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -407,9 +347,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The molecule N50 for all molecules that
-are ≥ 150 kbp in length
- INTEGER</t>
+          <t>INTEGER</t>
         </r>
       </text>
     </comment>
@@ -422,9 +360,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The molecule N50 for all molecules that
-are ≥ 20 kbp in length
- INTEGER</t>
+          <t>INTEGER</t>
         </r>
       </text>
     </comment>
@@ -437,9 +373,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The average number of fluorescent labels
-per unit length of DNA
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -452,10 +386,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Map rate (%) is the percentage of
-sequencing reads that successfully align
-to a reference genome.
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -468,11 +399,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The percentage of labeled sites whose
-observed positions differ from the
-expected positions in the reference
-genome
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -485,10 +412,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>The percentage of expected label sites
-from the reference genome that are
-missing in the observed DNA molecules
- DECIMAL</t>
+          <t>DECIMAL</t>
         </r>
       </text>
     </comment>
@@ -501,22 +425,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Other NGS quality control metrics,
-including but not limited to (i)
-sequencer metrics such as yield, error
-rate, density (K/mm2), cluster PF (%)
-and phas/prephas (%), (ii) alignment
-metrics such as QM insert size, GC
-content, QM duplicated reads (%), QM
-error rate, uniformity/evenness of
-coverage and maternal cell
-contamination, and (iii) variant call
-metrics such as number of SNVs/CNVs/SVs
-called, number of missense/nonsense
-variants, common variants (%), unique
-variants (%), gender match and trio
-inheritance check
- TEXT</t>
+          <t>TEXT</t>
         </r>
       </text>
     </comment>
@@ -529,10 +438,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Analysis or reanalysis of existing data
-collected by another centre usually for
-a different purpose
- Select one or more items from
+          <t>Select one or more items from
 Organisations</t>
         </r>
       </text>
@@ -546,9 +452,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>A written explanation, observation or
-criticism added to textual material
- TEXT</t>
+          <t>TEXT</t>
         </r>
       </text>
     </comment>

</xml_diff>